<commit_message>
﻿Carga: cuatro responsables, uno por subdireccion
Renombra todos los responsables a un solo nombre por subdireccion para
que el panel "Carga por responsable" muestre exactamente cuatro tarjetas:

- Amanda — Subdireccion de Archivo (5 tareas)
- Fabiola — Subdireccion de Gestion de Obras Inducidas (6 tareas)
- Mario — Subdireccion de Procesos Administrativos de Construccion (7)
- Samanta — Enlace administrativo del Director (3)

Aplica en:
- USUARIOS: nombre e iniciales de cada capturista (Amanda/AM, Fabiola/FA,
  Mario/MA, Samanta/SM).
- TAREAS: el campo responsable de las 21 tareas se reemplaza por el
  nombre asignado a su subdireccion.
- generar-plantillas.js: misma lista de nombres en los ejemplos.
- Plantillas .xlsx (5 archivos): regeneradas para reflejar los cambios.

validado_por sigue siendo Ing. Adrian Tavares (el Director).
</commit_message>
<xml_diff>
--- a/Plantilla-TT-Consolidada.xlsx
+++ b/Plantilla-TT-Consolidada.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="80">
   <si>
     <t>ATTRAPI · TT — Vista Consolidada · Cuatro Subdirecciones</t>
   </si>
@@ -52,7 +52,7 @@
     <t>SA-001</t>
   </si>
   <si>
-    <t>M. Hernández</t>
+    <t>Amanda</t>
   </si>
   <si>
     <t>Transferencia primaria expediente 2024 obras inducidas</t>
@@ -91,9 +91,6 @@
     <t>SA-003</t>
   </si>
   <si>
-    <t>P. Martínez</t>
-  </si>
-  <si>
     <t>Solicitud de baja documental ejercicios 2018-2019</t>
   </si>
   <si>
@@ -112,7 +109,7 @@
     <t>SGOI-001</t>
   </si>
   <si>
-    <t>J. López</t>
+    <t>Fabiola</t>
   </si>
   <si>
     <t>Reubicación líneas CFE km 42+300 Tramo II Querétaro-Irapuato</t>
@@ -130,9 +127,6 @@
     <t>SGOI-002</t>
   </si>
   <si>
-    <t>R. Domínguez</t>
-  </si>
-  <si>
     <t>Liberación derecho de vía Salinas Victoria NL</t>
   </si>
   <si>
@@ -148,9 +142,6 @@
     <t>SGOI-006</t>
   </si>
   <si>
-    <t>A. Ortiz</t>
-  </si>
-  <si>
     <t>Reporte mensual obras inducidas abril 2026</t>
   </si>
   <si>
@@ -169,7 +160,7 @@
     <t>SPAC-001</t>
   </si>
   <si>
-    <t>R. Sánchez</t>
+    <t>Mario</t>
   </si>
   <si>
     <t>Formalización contrato segmento 15A1 Saltillo-N. Laredo</t>
@@ -187,9 +178,6 @@
     <t>SPAC-002</t>
   </si>
   <si>
-    <t>J. R. García</t>
-  </si>
-  <si>
     <t>Acto de fallo segmento 15A2 Saltillo-N. Laredo</t>
   </si>
   <si>
@@ -223,7 +211,7 @@
     <t>ENLACE-001</t>
   </si>
   <si>
-    <t>Lic. C. Méndez</t>
+    <t>Samanta</t>
   </si>
   <si>
     <t>Compilación de acuerdos del Comité Directivo abril 2026</t>
@@ -961,19 +949,19 @@
         <v>25</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>30</v>
       </c>
       <c r="H6" s="8">
         <v>46203.25</v>
@@ -984,25 +972,25 @@
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="H7" s="11">
         <v>46203.25</v>
@@ -1013,25 +1001,25 @@
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="F8" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>43</v>
       </c>
       <c r="H8" s="8">
         <v>46172.25</v>
@@ -1042,25 +1030,25 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>46</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="H9" s="11">
         <v>46149.25</v>
@@ -1071,25 +1059,25 @@
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="E10" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="F10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>56</v>
       </c>
       <c r="H10" s="8">
         <v>46152.25</v>
@@ -1100,25 +1088,25 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B11" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>62</v>
       </c>
       <c r="H11" s="11">
         <v>46129.25</v>
@@ -1129,25 +1117,25 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B12" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="H12" s="8">
         <v>46149.25</v>
@@ -1158,25 +1146,25 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="F13" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="G13" s="10" t="s">
         <v>70</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>74</v>
       </c>
       <c r="H13" s="11">
         <v>46157.25</v>
@@ -1187,25 +1175,25 @@
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>75</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>79</v>
       </c>
       <c r="H14" s="8">
         <v>46149.25</v>
@@ -1216,25 +1204,25 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>72</v>
-      </c>
       <c r="F15" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H15" s="11">
         <v>46142.25</v>

</xml_diff>

<commit_message>
﻿Nombres en MAYUSCULAS: AMANDA, FABIOLA, MARIO, SAMANTA
Aplicado en:
- USUARIOS.nombre (lo que muestra el avatar y el saludo).
- TAREAS.responsable de las 21 tareas (lo que se ve en tarjetas y modal).
- generar-plantillas.js (responsable en filas de ejemplo de los xlsx).
- 5 plantillas .xlsx regeneradas.
</commit_message>
<xml_diff>
--- a/Plantilla-TT-Consolidada.xlsx
+++ b/Plantilla-TT-Consolidada.xlsx
@@ -55,7 +55,7 @@
     <t>SA-001</t>
   </si>
   <si>
-    <t>Amanda</t>
+    <t>AMANDA</t>
   </si>
   <si>
     <t>Transferencia primaria expediente 2024 obras inducidas</t>
@@ -118,7 +118,7 @@
     <t>SGOI-001</t>
   </si>
   <si>
-    <t>Fabiola</t>
+    <t>FABIOLA</t>
   </si>
   <si>
     <t>Reubicación líneas CFE km 42+300 Tramo II Querétaro-Irapuato</t>
@@ -169,7 +169,7 @@
     <t>SPAC-001</t>
   </si>
   <si>
-    <t>Mario</t>
+    <t>MARIO</t>
   </si>
   <si>
     <t>Formalización contrato segmento 15A1 Saltillo-N. Laredo</t>
@@ -220,7 +220,7 @@
     <t>ENLACE-001</t>
   </si>
   <si>
-    <t>Samanta</t>
+    <t>SAMANTA</t>
   </si>
   <si>
     <t>Compilación de acuerdos del Comité Directivo abril 2026</t>

</xml_diff>